<commit_message>
feat: externalize dispatcher configuration and standardize logging
</commit_message>
<xml_diff>
--- a/config/Config.xlsx
+++ b/config/Config.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Programming Projects\uipath-order-intake-validator\config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8A29DCD3-7694-4480-93A9-E761ACE4BD6E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8FEF63CB-F1CA-4966-A83E-3EBE52A81331}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="25">
   <si>
     <t>Name</t>
   </si>
@@ -57,9 +57,6 @@
     <t>InputFilePath</t>
   </si>
   <si>
-    <t>....\input\sample_orders.xlsx</t>
-  </si>
-  <si>
     <t>Dispatcher input file</t>
   </si>
   <si>
@@ -91,6 +88,18 @@
   </si>
   <si>
     <t>Supported countries</t>
+  </si>
+  <si>
+    <t>ComponentName</t>
+  </si>
+  <si>
+    <t>Dispatcher</t>
+  </si>
+  <si>
+    <t>Component writing the logs</t>
+  </si>
+  <si>
+    <t>..\..\input\sample_orders.xlsx</t>
   </si>
 </sst>
 </file>
@@ -422,7 +431,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C8"/>
+  <dimension ref="A1:C9"/>
   <sheetFormatPr defaultColWidth="79" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="18.109375" bestFit="1" customWidth="1"/>
@@ -468,54 +477,65 @@
         <v>9</v>
       </c>
       <c r="B4" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="C4" s="2" t="s">
         <v>10</v>
-      </c>
-      <c r="C4" s="2" t="s">
-        <v>11</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="B5" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="B5" s="2" t="s">
+      <c r="C5" s="2" t="s">
         <v>13</v>
-      </c>
-      <c r="C5" s="2" t="s">
-        <v>14</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B6" s="2">
         <v>1</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7" s="2" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B7" s="2">
         <v>1</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A8" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="B8" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="B8" s="2" t="s">
+      <c r="C8" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="C8" s="2" t="s">
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A9" s="2" t="s">
         <v>21</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>23</v>
       </c>
     </row>
   </sheetData>

</xml_diff>